<commit_message>
Implemented leave entity changes and DTO classes
</commit_message>
<xml_diff>
--- a/Documentation/Site Maps/Modules/Leave Management/Leave request types.xlsx
+++ b/Documentation/Site Maps/Modules/Leave Management/Leave request types.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\NET Projects\KEN Solutions\KenHRApp\Documentation\Site Maps\Modules\Leave Management\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\NET Projects\ebrosas\KENSolutions\Documentation\Site Maps\Modules\Leave Management\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36FB4EEA-E613-497F-9BD4-723BE3F6FFDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A886549F-7013-469B-B37B-F7E27F0164D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="19440" windowHeight="15000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Leave Types" sheetId="1" r:id="rId1"/>

</xml_diff>